<commit_message>
Update adversarial gpt-4o evaluation to full 152-prompt set
The adversarial gpt-4o run now covers all 152 prompts (previously 134),
matching the CodeLlama run. Attack success rate 10.61 percent to 0.00 percent
(McNemar p=0.000512). Evidence spreadsheets regenerated accordingly.
</commit_message>
<xml_diff>
--- a/results/excels/evaluation_results.xlsx
+++ b/results/excels/evaluation_results.xlsx
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>286</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3">
@@ -898,7 +898,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>11.40%</t>
+          <t>10.61%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>11.40%</t>
+          <t>10.61%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>6.06%</t>
+          <t>8.33%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>7.02%</t>
+          <t>4.55%</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">

</xml_diff>